<commit_message>
feat(F-NAR-016): TREE-DIF-045 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-045.xlsx
+++ b/stories/arbres/TREE-DIF-045.xlsx
@@ -4267,12 +4267,12 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse, puis s'arrête. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Le bleu garde une goutte, tout au fond. Toc. Une bulle se tait, puis l'autre. L'évier redevient calme, autour du bac.</t>
+          <t>Le bleu rejoint le bac, encore mouillé. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Le bleu garde une goutte, tout au fond. Toc. Une bulle se tait, puis l'autre. L'évier reste calme, derrière eux.</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse, puis s'arrête. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Le bleu garde une goutte, tout au fond. Toc. Une bulle se tait, puis l'autre. L'évier redevient calme, autour du bac.</t>
+          <t>Le bleu rejoint le bac, encore mouillé. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Le bleu garde une goutte, tout au fond. Toc. Une bulle se tait, puis l'autre. L'évier reste calme, derrière eux.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -4407,14 +4407,14 @@
       <c r="AV19" s="2" t="inlineStr"/>
       <c r="AW19" t="inlineStr">
         <is>
-          <t>narrateur|Une goutte glisse, puis s'arrête.
+          <t>narrateur|Le bleu rejoint le bac, encore mouillé.
 copine|On a attendu l'eau.
 papa|Le savon n'a plus pris vos bras.
 maman|Rentrez le torchon, après le bac.
 narrateur|Le bleu garde une goutte, tout au fond.
 enfant-m|Toc.
 narrateur|Une bulle se tait, puis l'autre.
-narrateur|L'évier redevient calme, autour du bac.</t>
+narrateur|L'évier reste calme, derrière eux.</t>
         </is>
       </c>
     </row>
@@ -4615,12 +4615,12 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient le galet, tout net. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Le bleu garde une goutte, tout au fond. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. L'eau sent encore le savon tiède.</t>
+          <t>Le filet pose le galet au fond du bac. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Le bleu garde une goutte, tout au fond. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient le galet, tout net. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Le bleu garde une goutte, tout au fond. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. L'eau sent encore le savon tiède.</t>
+          <t>Le filet pose le galet au fond du bac. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Le bleu garde une goutte, tout au fond. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -4755,14 +4755,14 @@
       <c r="AV21" s="2" t="inlineStr"/>
       <c r="AW21" t="inlineStr">
         <is>
-          <t>narrateur|Le filet tient le galet, tout net.
+          <t>narrateur|Le filet pose le galet au fond du bac.
 copine|On tenait, tous les deux.
 papa|Je remporte l'épuisette, tout à l'heure.
 maman|Le poisson vous attend.
 narrateur|Le bleu garde une goutte, tout au fond.
 narrateur|Aniss essuie une main sur son pantalon.
 narrateur|Un grain de craie reste sur le filet.
-narrateur|L'eau sent encore le savon tiède.</t>
+narrateur|Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
     </row>
@@ -4963,12 +4963,12 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le bleu descendre. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Le bleu garde une goutte, tout au fond. Aniss pose un doigt sur le robinet. Il bouge, tout petit. Un rai de soleil barre encore l'évier.</t>
+          <t>Les mains d'Aniss laissent le bleu au fond du bac. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Le bleu garde une goutte, tout au fond. Aniss pose un doigt sur le verre. Une bulle bouge, toute petite. Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le bleu descendre. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Le bleu garde une goutte, tout au fond. Aniss pose un doigt sur le robinet. Il bouge, tout petit. Un rai de soleil barre encore l'évier.</t>
+          <t>Les mains d'Aniss laissent le bleu au fond du bac. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Le bleu garde une goutte, tout au fond. Aniss pose un doigt sur le verre. Une bulle bouge, toute petite. Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
@@ -5103,14 +5103,14 @@
       <c r="AV23" s="2" t="inlineStr"/>
       <c r="AW23" t="inlineStr">
         <is>
-          <t>narrateur|Les mains d'Aniss laissent le bleu descendre.
+          <t>narrateur|Les mains d'Aniss laissent le bleu au fond du bac.
 copine|C'était plus facile, là.
 papa|Tes bras ont guidé le galet.
 maman|Le fond gardera son ombre.
 narrateur|Le bleu garde une goutte, tout au fond.
-narrateur|Aniss pose un doigt sur le robinet.
-narrateur|Il bouge, tout petit.
-narrateur|Un rai de soleil barre encore l'évier.</t>
+narrateur|Aniss pose un doigt sur le verre.
+narrateur|Une bulle bouge, toute petite.
+narrateur|Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
     </row>
@@ -9240,12 +9240,12 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse, puis s'arrête. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. L'épuisette sent encore l'eau tiède. Toc. Une bulle se tait, puis l'autre. L'évier redevient calme, autour du bac.</t>
+          <t>Le bleu rejoint le bac, encore mouillé. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. L'épuisette sent encore l'eau tiède. Toc. Une bulle se tait, puis l'autre. L'évier reste calme, derrière eux.</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse, puis s'arrête. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. L'épuisette sent encore l'eau tiède. Toc. Une bulle se tait, puis l'autre. L'évier redevient calme, autour du bac.</t>
+          <t>Le bleu rejoint le bac, encore mouillé. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. L'épuisette sent encore l'eau tiède. Toc. Une bulle se tait, puis l'autre. L'évier reste calme, derrière eux.</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -9380,14 +9380,14 @@
       <c r="AV47" s="2" t="inlineStr"/>
       <c r="AW47" t="inlineStr">
         <is>
-          <t>narrateur|Une goutte glisse, puis s'arrête.
+          <t>narrateur|Le bleu rejoint le bac, encore mouillé.
 copine|On a attendu l'eau.
 papa|Le savon n'a plus pris vos bras.
 maman|Rentrez le torchon, après le bac.
 narrateur|L'épuisette sent encore l'eau tiède.
 enfant-m|Toc.
 narrateur|Une bulle se tait, puis l'autre.
-narrateur|L'évier redevient calme, autour du bac.</t>
+narrateur|L'évier reste calme, derrière eux.</t>
         </is>
       </c>
     </row>
@@ -9588,12 +9588,12 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient le galet, tout net. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. L'épuisette sent encore l'eau tiède. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. L'eau sent encore le savon tiède.</t>
+          <t>Le filet pose le galet au fond du bac. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. L'épuisette sent encore l'eau tiède. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient le galet, tout net. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. L'épuisette sent encore l'eau tiède. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. L'eau sent encore le savon tiède.</t>
+          <t>Le filet pose le galet au fond du bac. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. L'épuisette sent encore l'eau tiède. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
@@ -9728,14 +9728,14 @@
       <c r="AV49" s="2" t="inlineStr"/>
       <c r="AW49" t="inlineStr">
         <is>
-          <t>narrateur|Le filet tient le galet, tout net.
+          <t>narrateur|Le filet pose le galet au fond du bac.
 copine|On tenait, tous les deux.
 papa|Je remporte l'épuisette, tout à l'heure.
 maman|Le poisson vous attend.
 narrateur|L'épuisette sent encore l'eau tiède.
 narrateur|Aniss essuie une main sur son pantalon.
 narrateur|Un grain de craie reste sur le filet.
-narrateur|L'eau sent encore le savon tiède.</t>
+narrateur|Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
     </row>
@@ -9936,12 +9936,12 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le bleu descendre. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. L'épuisette sent encore l'eau tiède. Aniss pose un doigt sur le robinet. Il bouge, tout petit. Un rai de soleil barre encore l'évier.</t>
+          <t>Les mains d'Aniss laissent le bleu au fond du bac. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. L'épuisette sent encore l'eau tiède. Aniss pose un doigt sur le verre. Une bulle bouge, toute petite. Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le bleu descendre. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. L'épuisette sent encore l'eau tiède. Aniss pose un doigt sur le robinet. Il bouge, tout petit. Un rai de soleil barre encore l'évier.</t>
+          <t>Les mains d'Aniss laissent le bleu au fond du bac. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. L'épuisette sent encore l'eau tiède. Aniss pose un doigt sur le verre. Une bulle bouge, toute petite. Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -10076,14 +10076,14 @@
       <c r="AV51" s="2" t="inlineStr"/>
       <c r="AW51" t="inlineStr">
         <is>
-          <t>narrateur|Les mains d'Aniss laissent le bleu descendre.
+          <t>narrateur|Les mains d'Aniss laissent le bleu au fond du bac.
 copine|C'était plus facile, là.
 papa|Tes bras ont guidé le galet.
 maman|Le fond gardera son ombre.
 narrateur|L'épuisette sent encore l'eau tiède.
-narrateur|Aniss pose un doigt sur le robinet.
-narrateur|Il bouge, tout petit.
-narrateur|Un rai de soleil barre encore l'évier.</t>
+narrateur|Aniss pose un doigt sur le verre.
+narrateur|Une bulle bouge, toute petite.
+narrateur|Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
     </row>
@@ -14213,12 +14213,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse, puis s'arrête. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Un carreau de torchon reste un peu humide. Toc. Une bulle se tait, puis l'autre. L'évier redevient calme, autour du bac.</t>
+          <t>Le bleu rejoint le bac, encore mouillé. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Un carreau de torchon reste un peu humide. Toc. Une bulle se tait, puis l'autre. L'évier reste calme, derrière eux.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Une goutte glisse, puis s'arrête. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Un carreau de torchon reste un peu humide. Toc. Une bulle se tait, puis l'autre. L'évier redevient calme, autour du bac.</t>
+          <t>Le bleu rejoint le bac, encore mouillé. On a attendu l'eau. Le savon n'a plus pris vos bras. Rentrez le torchon, après le bac. Un carreau de torchon reste un peu humide. Toc. Une bulle se tait, puis l'autre. L'évier reste calme, derrière eux.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -14353,14 +14353,14 @@
       <c r="AV75" s="2" t="inlineStr"/>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>narrateur|Une goutte glisse, puis s'arrête.
+          <t>narrateur|Le bleu rejoint le bac, encore mouillé.
 copine|On a attendu l'eau.
 papa|Le savon n'a plus pris vos bras.
 maman|Rentrez le torchon, après le bac.
 narrateur|Un carreau de torchon reste un peu humide.
 enfant-m|Toc.
 narrateur|Une bulle se tait, puis l'autre.
-narrateur|L'évier redevient calme, autour du bac.</t>
+narrateur|L'évier reste calme, derrière eux.</t>
         </is>
       </c>
     </row>
@@ -14561,12 +14561,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient le galet, tout net. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Un carreau de torchon reste un peu humide. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. L'eau sent encore le savon tiède.</t>
+          <t>Le filet pose le galet au fond du bac. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Un carreau de torchon reste un peu humide. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>Le filet tient le galet, tout net. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Un carreau de torchon reste un peu humide. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. L'eau sent encore le savon tiède.</t>
+          <t>Le filet pose le galet au fond du bac. On tenait, tous les deux. Je remporte l'épuisette, tout à l'heure. Le poisson vous attend. Un carreau de torchon reste un peu humide. Aniss essuie une main sur son pantalon. Un grain de craie reste sur le filet. Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr">
@@ -14701,14 +14701,14 @@
       <c r="AV77" s="2" t="inlineStr"/>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>narrateur|Le filet tient le galet, tout net.
+          <t>narrateur|Le filet pose le galet au fond du bac.
 copine|On tenait, tous les deux.
 papa|Je remporte l'épuisette, tout à l'heure.
 maman|Le poisson vous attend.
 narrateur|Un carreau de torchon reste un peu humide.
 narrateur|Aniss essuie une main sur son pantalon.
 narrateur|Un grain de craie reste sur le filet.
-narrateur|L'eau sent encore le savon tiède.</t>
+narrateur|Le verre sent encore l'eau tiède.</t>
         </is>
       </c>
     </row>
@@ -14909,12 +14909,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le bleu descendre. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Un carreau de torchon reste un peu humide. Aniss pose un doigt sur le robinet. Il bouge, tout petit. Un rai de soleil barre encore l'évier.</t>
+          <t>Les mains d'Aniss laissent le bleu au fond du bac. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Un carreau de torchon reste un peu humide. Aniss pose un doigt sur le verre. Une bulle bouge, toute petite. Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>Les mains d'Aniss laissent le bleu descendre. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Un carreau de torchon reste un peu humide. Aniss pose un doigt sur le robinet. Il bouge, tout petit. Un rai de soleil barre encore l'évier.</t>
+          <t>Les mains d'Aniss laissent le bleu au fond du bac. C'était plus facile, là. Tes bras ont guidé le galet. Le fond gardera son ombre. Un carreau de torchon reste un peu humide. Aniss pose un doigt sur le verre. Une bulle bouge, toute petite. Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr">
@@ -15049,14 +15049,14 @@
       <c r="AV79" s="2" t="inlineStr"/>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>narrateur|Les mains d'Aniss laissent le bleu descendre.
+          <t>narrateur|Les mains d'Aniss laissent le bleu au fond du bac.
 copine|C'était plus facile, là.
 papa|Tes bras ont guidé le galet.
 maman|Le fond gardera son ombre.
 narrateur|Un carreau de torchon reste un peu humide.
-narrateur|Aniss pose un doigt sur le robinet.
-narrateur|Il bouge, tout petit.
-narrateur|Un rai de soleil barre encore l'évier.</t>
+narrateur|Aniss pose un doigt sur le verre.
+narrateur|Une bulle bouge, toute petite.
+narrateur|Un rai de soleil barre encore le bac.</t>
         </is>
       </c>
     </row>
@@ -16489,7 +16489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -16539,6 +16539,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>